<commit_message>
Atualização automática das bases ECODATA
</commit_message>
<xml_diff>
--- a/data/final/bcb_sgs/base_bcb_sgs_mensal_larga.xlsx
+++ b/data/final/bcb_sgs/base_bcb_sgs_mensal_larga.xlsx
@@ -615,10 +615,10 @@
         <v>6.25</v>
       </c>
       <c r="C2" t="n">
-        <v>0.021182</v>
+        <v>0.021256</v>
       </c>
       <c r="D2" t="n">
-        <v>0.021182</v>
+        <v>0.021256</v>
       </c>
       <c r="E2" t="n">
         <v>1.16</v>
@@ -773,10 +773,10 @@
         <v>1.5</v>
       </c>
       <c r="AF3" t="n">
-        <v>0.003062</v>
+        <v>0.002988</v>
       </c>
       <c r="AG3" t="n">
-        <v>0.003062</v>
+        <v>0.002988</v>
       </c>
       <c r="AH3" t="n">
         <v>-0.01</v>

</xml_diff>